<commit_message>
Add backend calculation engine for graph data
- Excel data extraction with formula steps

- Dynamic placeholder expansion

- Numeric processing and error handling

Visualization layer not included in this commit.
</commit_message>
<xml_diff>
--- a/backend/Rwanda/technoeconomic-inputs-CleanStep.xlsx
+++ b/backend/Rwanda/technoeconomic-inputs-CleanStep.xlsx
@@ -1445,40 +1445,40 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E2" s="8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H2" s="8" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I2" s="8" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J2" s="8" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K2" s="8" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L2" s="8" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="M2" s="8" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="N2" s="8" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -1613,40 +1613,40 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>0.09441198237754599</v>
+        <v>0.09</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>0.1791091825492832</v>
+        <v>0.18</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>0.1773180907237903</v>
+        <v>0.18</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.1755449098165524</v>
+        <v>0.18</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>0.1737894607183869</v>
+        <v>0.17</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>0.1720515661112031</v>
+        <v>0.17</v>
       </c>
       <c r="I5" s="8" t="n">
-        <v>0.1300782577475552</v>
+        <v>0.13</v>
       </c>
       <c r="J5" s="8" t="n">
-        <v>0.08872645212259944</v>
+        <v>0.09</v>
       </c>
       <c r="K5" s="8" t="n">
-        <v>0.08783918760137345</v>
+        <v>0.09</v>
       </c>
       <c r="L5" s="8" t="n">
-        <v>0.0869607957253597</v>
+        <v>0.09</v>
       </c>
       <c r="M5" s="8" t="n">
-        <v>0.08609118776810612</v>
+        <v>0.09</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>0.07967632839653764</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="6">
@@ -1709,40 +1709,40 @@
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>4.32143283622375</v>
+        <v>4.32</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>6.236309089950275</v>
+        <v>6.24</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>8.821590307560108</v>
+        <v>8.82</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>11.35454226990875</v>
+        <v>11.35</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>13.83595303397966</v>
+        <v>13.84</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>16.26660012854216</v>
+        <v>16.27</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>18.64725068591002</v>
+        <v>18.65</v>
       </c>
       <c r="J7" s="8" t="n">
-        <v>19.39869399949082</v>
+        <v>19.4</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>19.74037768502499</v>
+        <v>19.74</v>
       </c>
       <c r="L7" s="8" t="n">
-        <v>20.07328782744852</v>
+        <v>20.07</v>
       </c>
       <c r="M7" s="8" t="n">
-        <v>20.39756572925508</v>
+        <v>20.4</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>20.71335074424277</v>
+        <v>20.71</v>
       </c>
     </row>
     <row r="8">
@@ -1759,38 +1759,60 @@
       <c r="C8" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="D8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="10" t="n">
-        <v>0</v>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>